<commit_message>
interest_rt: rename a/b to beta/margin_pct, fix client caps
- interest_rt.xlsx: a -> beta, b -> margin_pct (clearer for business users;
  "b" was easy to mistake for beta). All readers updated.
- client_cap is a decimal, so 0.1 meant 10%, not the intended 0.1%:
  6300 cap -> 0.001; 6000 cap removed (beta=margin=0, so it never binds).
- Deposit generation now applies client_cap (previously only NII/EVE did)
  and treats a blank margin_pct as 0 -- 6300 had client_rt NULL on every row.
- Docs: new column names, index comes from bank_data.xlsx rate_index,
  floors/caps are decimals.
- Regenerated pipeline outputs and app caches (incl. ftp_rates.npz).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance_generate/input_data/interest_rt.xlsx
+++ b/balance_generate/input_data/interest_rt.xlsx
@@ -423,12 +423,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>margin_pct</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -465,9 +465,6 @@
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="n">
-        <v>0.1</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -630,11 +627,14 @@
       <c r="B14" t="n">
         <v>0.1</v>
       </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="15">

</xml_diff>